<commit_message>
feat: Adiciona processamento do arquivo 'CONTROLES POR COMISSÃO E GESTORES.xlsx' para unificar dados de gestor e fiscal, incluindo a nova coluna 'FISCAL' e ajustando a precisão de valores numéricos.
</commit_message>
<xml_diff>
--- a/ANALITICA.xlsx
+++ b/ANALITICA.xlsx
@@ -4468,16 +4468,16 @@
         <v>231</v>
       </c>
       <c r="G55" s="11">
-        <v>0.9702</v>
+        <v>0.9754</v>
       </c>
       <c r="H55" s="12">
         <v>56189486.28</v>
       </c>
       <c r="I55" s="13">
-        <v>54515037.34</v>
+        <v>54809333.5</v>
       </c>
       <c r="J55" s="12">
-        <v>1674448.9399999976</v>
+        <v>1380152.7800000012</v>
       </c>
       <c r="K55" s="14">
         <v>45035</v>
@@ -5342,16 +5342,16 @@
         <v>318</v>
       </c>
       <c r="G78" s="11">
-        <v>0</v>
+        <v>0.0134</v>
       </c>
       <c r="H78" s="12">
         <v>4705907.3</v>
       </c>
       <c r="I78" s="13">
-        <v>0</v>
+        <v>63006.28</v>
       </c>
       <c r="J78" s="12">
-        <v>4705907.3</v>
+        <v>4642901.02</v>
       </c>
       <c r="K78" s="14">
         <v>46009</v>

</xml_diff>

<commit_message>
Renamed 'RELACAO DE TODAS AS OBRAS DA SECRETARIA.xlsx' to 'TODAS AS OBRAS DA SECRETARIA.xlsx' and updated associated measurement spreadsheets.
</commit_message>
<xml_diff>
--- a/ANALITICA.xlsx
+++ b/ANALITICA.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="638">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1031" uniqueCount="641">
   <si>
     <t>Municipio</t>
   </si>
@@ -1740,6 +1740,15 @@
   </si>
   <si>
     <t>RECUPERAÇÃO DE EQUIPAMENTOS DO TELEFÉRICO DO ALEMÃO - RJ</t>
+  </si>
+  <si>
+    <t>330001/001152/2025</t>
+  </si>
+  <si>
+    <t>CONTRATAÇÃO DE UMA EMPRESA ESPECIALIZADA NA EXECUÇÃO DE SERVIÇOS DE ESTABILIZAÇÃO DE SOLOS COM ESTABILIZADOR IÔNICO LÍQUIDO, COM PROPRIEDADES DE AUMENTO DA RESISTÊNCIA DO SOLO E RESISTÊNCIA À ÁGUA, 100% AMBIENTALMENTE SUSTENTÁVEL, MONOCOMPONENTE, APLICADO IN SITU, COM O FORNECIMENTO DE TODOS OS EQUIPAMENTOS, MAQUINÁRIO, MÃO DE OBRA E TODOS OS MATERIAIS NECESSÁRIOS PARA CADA TIPO DE SERVIÇO, CONFORME AS CONDIÇÕES E EXIGÊNCIAS ESTABELECIDAS.</t>
+  </si>
+  <si>
+    <t>Não existe na tabela Contratadas</t>
   </si>
   <si>
     <t>São Francisco de Itabapoana</t>
@@ -1936,7 +1945,7 @@
     <numFmt numFmtId="164" formatCode="R$#,##0.00;-R$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="DD-MM-YYYY"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1946,7 +1955,11 @@
     </font>
     <font>
       <color rgb="FF404040"/>
-      <sz val="13"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <color rgb="FF404040"/>
+      <sz val="15"/>
     </font>
   </fonts>
   <fills count="4">
@@ -2021,20 +2034,20 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2391,21 +2404,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L169"/>
+  <dimension ref="A1:L170"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="16.46153846153846" style="1" customWidth="1"/>
-    <col min="2" max="2" width="23.571428571428573" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.153846153846153" style="1" customWidth="1"/>
-    <col min="5" max="5" width="36.15384615384615" style="1" customWidth="1"/>
-    <col min="6" max="6" width="33.07692307692308" style="1" customWidth="1"/>
+    <col min="1" max="1" width="18" style="1" customWidth="1"/>
+    <col min="2" max="2" width="25" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.76923076923077" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.384615384615383" style="1" customWidth="1"/>
+    <col min="5" max="5" width="41.07692307692308" style="1" customWidth="1"/>
+    <col min="6" max="6" width="36.15384615384615" style="1" customWidth="1"/>
     <col min="7" max="7" width="18.76923076923077" style="1" customWidth="1"/>
     <col min="8" max="8" width="21.23076923076923" style="2" customWidth="1"/>
     <col min="9" max="9" width="20.76923076923077" style="3" customWidth="1"/>
     <col min="10" max="10" width="19.846153846153847" style="2" customWidth="1"/>
-    <col min="11" max="11" width="18.92857142857143" style="4" customWidth="1"/>
-    <col min="12" max="12" width="15.214285714285715" style="4" customWidth="1"/>
+    <col min="11" max="11" width="16.923076923076923" style="4" customWidth="1"/>
+    <col min="12" max="12" width="16.615384615384617" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -3682,16 +3695,16 @@
         <v>154</v>
       </c>
       <c r="G34" s="11">
-        <v>0.5958</v>
+        <v>0.7181000000000001</v>
       </c>
       <c r="H34" s="12">
         <v>6016602.48</v>
       </c>
       <c r="I34" s="13">
-        <v>3584685.32</v>
+        <v>4320723.47</v>
       </c>
       <c r="J34" s="12">
-        <v>2431917.1600000006</v>
+        <v>1695879.0100000007</v>
       </c>
       <c r="K34" s="14">
         <v>45133</v>
@@ -4153,7 +4166,7 @@
         <v>44753</v>
       </c>
       <c r="L46" s="14">
-        <v>46077</v>
+        <v>46443</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
@@ -5647,7 +5660,7 @@
         <v>347</v>
       </c>
       <c r="D86" s="11" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="E86" s="11" t="s">
         <v>348</v>
@@ -6910,16 +6923,16 @@
         <v>45</v>
       </c>
       <c r="G119" s="11">
-        <v>0.0165</v>
+        <v>0.0321</v>
       </c>
       <c r="H119" s="12">
         <v>7430869.32</v>
       </c>
       <c r="I119" s="13">
-        <v>122778.19</v>
+        <v>238550.07</v>
       </c>
       <c r="J119" s="12">
-        <v>7308091.13</v>
+        <v>7192319.25</v>
       </c>
       <c r="K119" s="14">
         <v>45865</v>
@@ -8184,83 +8197,81 @@
     </row>
     <row r="153" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A153" s="11" t="s">
+        <v>510</v>
+      </c>
+      <c r="B153" s="11" t="s">
         <v>576</v>
       </c>
-      <c r="B153" s="11" t="s">
+      <c r="C153" s="11"/>
+      <c r="D153" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="E153" s="11" t="s">
         <v>577</v>
       </c>
-      <c r="C153" s="11" t="s">
+      <c r="F153" s="11" t="s">
         <v>578</v>
       </c>
-      <c r="D153" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="E153" s="11" t="s">
-        <v>579</v>
-      </c>
-      <c r="F153" s="11" t="s">
-        <v>580</v>
-      </c>
       <c r="G153" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H153" s="12">
-        <v>10061005.41</v>
+        <v>201720000</v>
       </c>
       <c r="I153" s="13">
-        <v>10061005.39</v>
+        <v>0</v>
       </c>
       <c r="J153" s="12">
-        <v>0.019999999552965164</v>
-      </c>
-      <c r="K153" s="14">
-        <v>45261</v>
-      </c>
-      <c r="L153" s="14">
-        <v>45833</v>
+        <v>201720000</v>
+      </c>
+      <c r="K153" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="L153" s="15" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="154" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A154" s="11" t="s">
+        <v>579</v>
+      </c>
+      <c r="B154" s="11" t="s">
+        <v>580</v>
+      </c>
+      <c r="C154" s="11" t="s">
         <v>581</v>
       </c>
-      <c r="B154" s="11" t="s">
+      <c r="D154" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E154" s="11" t="s">
         <v>582</v>
       </c>
-      <c r="C154" s="11" t="s">
+      <c r="F154" s="11" t="s">
         <v>583</v>
-      </c>
-      <c r="D154" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="E154" s="11" t="s">
-        <v>584</v>
-      </c>
-      <c r="F154" s="11" t="s">
-        <v>45</v>
       </c>
       <c r="G154" s="11">
         <v>1</v>
       </c>
       <c r="H154" s="12">
-        <v>81950979.23</v>
+        <v>10061005.41</v>
       </c>
       <c r="I154" s="13">
-        <v>81950979</v>
+        <v>10061005.39</v>
       </c>
       <c r="J154" s="12">
-        <v>0.23000000417232513</v>
+        <v>0.019999999552965164</v>
       </c>
       <c r="K154" s="14">
-        <v>44792</v>
+        <v>45261</v>
       </c>
       <c r="L154" s="14">
-        <v>46022</v>
+        <v>45833</v>
       </c>
     </row>
     <row r="155" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A155" s="11" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="B155" s="11" t="s">
         <v>585</v>
@@ -8275,182 +8286,182 @@
         <v>587</v>
       </c>
       <c r="F155" s="11" t="s">
-        <v>588</v>
+        <v>45</v>
       </c>
       <c r="G155" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H155" s="12">
-        <v>41522873.42</v>
+        <v>81950979.23</v>
       </c>
       <c r="I155" s="13">
-        <v>0</v>
+        <v>81950979</v>
       </c>
       <c r="J155" s="12">
-        <v>41522873.42</v>
+        <v>0.23000000417232513</v>
       </c>
       <c r="K155" s="14">
-        <v>45901</v>
+        <v>44792</v>
       </c>
       <c r="L155" s="14">
-        <v>46801</v>
+        <v>46022</v>
       </c>
     </row>
     <row r="156" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A156" s="11" t="s">
+        <v>584</v>
+      </c>
+      <c r="B156" s="11" t="s">
+        <v>588</v>
+      </c>
+      <c r="C156" s="11" t="s">
         <v>589</v>
       </c>
-      <c r="B156" s="11" t="s">
+      <c r="D156" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E156" s="11" t="s">
         <v>590</v>
       </c>
-      <c r="C156" s="11" t="s">
+      <c r="F156" s="11" t="s">
         <v>591</v>
       </c>
-      <c r="D156" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="E156" s="11" t="s">
-        <v>592</v>
-      </c>
-      <c r="F156" s="11" t="s">
-        <v>323</v>
-      </c>
       <c r="G156" s="11">
-        <v>0.9728</v>
+        <v>0</v>
       </c>
       <c r="H156" s="12">
-        <v>4444784.22</v>
+        <v>41522873.42</v>
       </c>
       <c r="I156" s="13">
-        <v>4324004.81</v>
+        <v>0</v>
       </c>
       <c r="J156" s="12">
-        <v>120779.41000000015</v>
+        <v>41522873.42</v>
       </c>
       <c r="K156" s="14">
-        <v>45155</v>
+        <v>45901</v>
       </c>
       <c r="L156" s="14">
-        <v>45576</v>
+        <v>46801</v>
       </c>
     </row>
     <row r="157" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A157" s="11" t="s">
+        <v>592</v>
+      </c>
+      <c r="B157" s="11" t="s">
         <v>593</v>
       </c>
-      <c r="B157" s="11" t="s">
+      <c r="C157" s="11" t="s">
         <v>594</v>
       </c>
-      <c r="C157" s="11" t="s">
+      <c r="D157" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E157" s="11" t="s">
         <v>595</v>
       </c>
-      <c r="D157" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="E157" s="11" t="s">
-        <v>596</v>
-      </c>
       <c r="F157" s="11" t="s">
-        <v>111</v>
+        <v>323</v>
       </c>
       <c r="G157" s="11">
-        <v>0</v>
+        <v>0.9728</v>
       </c>
       <c r="H157" s="12">
-        <v>8995898.05</v>
+        <v>4444784.22</v>
       </c>
       <c r="I157" s="13">
-        <v>266299.23</v>
+        <v>4324004.81</v>
       </c>
       <c r="J157" s="12">
-        <v>8729598.82</v>
+        <v>120779.41000000015</v>
       </c>
       <c r="K157" s="14">
-        <v>44816</v>
+        <v>45155</v>
       </c>
       <c r="L157" s="14">
-        <v>44996</v>
+        <v>45576</v>
       </c>
     </row>
     <row r="158" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A158" s="11" t="s">
+        <v>596</v>
+      </c>
+      <c r="B158" s="11" t="s">
         <v>597</v>
       </c>
-      <c r="B158" s="11" t="s">
+      <c r="C158" s="11" t="s">
         <v>598</v>
       </c>
-      <c r="C158" s="11" t="s">
+      <c r="D158" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E158" s="11" t="s">
         <v>599</v>
       </c>
-      <c r="D158" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="E158" s="11" t="s">
-        <v>600</v>
-      </c>
       <c r="F158" s="11" t="s">
-        <v>580</v>
+        <v>111</v>
       </c>
       <c r="G158" s="11">
-        <v>0.3153</v>
+        <v>0</v>
       </c>
       <c r="H158" s="12">
-        <v>3294597.99</v>
+        <v>8995898.05</v>
       </c>
       <c r="I158" s="13">
-        <v>1038880.21</v>
+        <v>266299.23</v>
       </c>
       <c r="J158" s="12">
-        <v>2255717.7800000003</v>
+        <v>8729598.82</v>
       </c>
       <c r="K158" s="14">
-        <v>45278</v>
+        <v>44816</v>
       </c>
       <c r="L158" s="14">
-        <v>46122</v>
+        <v>44996</v>
       </c>
     </row>
     <row r="159" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A159" s="11" t="s">
+        <v>600</v>
+      </c>
+      <c r="B159" s="11" t="s">
         <v>601</v>
       </c>
-      <c r="B159" s="11" t="s">
+      <c r="C159" s="11" t="s">
         <v>602</v>
-      </c>
-      <c r="C159" s="11" t="s">
-        <v>603</v>
       </c>
       <c r="D159" s="11" t="s">
         <v>34</v>
       </c>
       <c r="E159" s="11" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="F159" s="11" t="s">
-        <v>505</v>
+        <v>583</v>
       </c>
       <c r="G159" s="11">
-        <v>0.9922</v>
+        <v>0.3153</v>
       </c>
       <c r="H159" s="12">
-        <v>6055289.34</v>
+        <v>3294597.99</v>
       </c>
       <c r="I159" s="13">
-        <v>6007931.02</v>
+        <v>1038880.21</v>
       </c>
       <c r="J159" s="12">
-        <v>47358.3200000003</v>
+        <v>2255717.7800000003</v>
       </c>
       <c r="K159" s="14">
-        <v>44715</v>
+        <v>45278</v>
       </c>
       <c r="L159" s="14">
-        <v>45075</v>
+        <v>46122</v>
       </c>
     </row>
     <row r="160" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A160" s="11" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="B160" s="11" t="s">
         <v>605</v>
@@ -8459,264 +8470,264 @@
         <v>606</v>
       </c>
       <c r="D160" s="11" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="E160" s="11" t="s">
         <v>607</v>
       </c>
       <c r="F160" s="11" t="s">
-        <v>45</v>
+        <v>505</v>
       </c>
       <c r="G160" s="11">
-        <v>0.22760000000000002</v>
+        <v>0.9922</v>
       </c>
       <c r="H160" s="12">
-        <v>8973983.87</v>
+        <v>6055289.34</v>
       </c>
       <c r="I160" s="13">
-        <v>2042159.29</v>
+        <v>6007931.02</v>
       </c>
       <c r="J160" s="12">
-        <v>6931824.579999999</v>
+        <v>47358.3200000003</v>
       </c>
       <c r="K160" s="14">
-        <v>44707</v>
+        <v>44715</v>
       </c>
       <c r="L160" s="14">
-        <v>45280</v>
+        <v>45075</v>
       </c>
     </row>
     <row r="161" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A161" s="11" t="s">
+        <v>604</v>
+      </c>
+      <c r="B161" s="11" t="s">
         <v>608</v>
       </c>
-      <c r="B161" s="11" t="s">
+      <c r="C161" s="11" t="s">
         <v>609</v>
       </c>
-      <c r="C161" s="11" t="s">
-        <v>249</v>
-      </c>
       <c r="D161" s="11" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E161" s="11" t="s">
         <v>610</v>
       </c>
       <c r="F161" s="11" t="s">
-        <v>149</v>
+        <v>45</v>
       </c>
       <c r="G161" s="11">
-        <v>1</v>
+        <v>0.22760000000000002</v>
       </c>
       <c r="H161" s="12">
-        <v>13792679.79</v>
+        <v>8973983.87</v>
       </c>
       <c r="I161" s="13">
-        <v>13792679.79</v>
+        <v>2042159.29</v>
       </c>
       <c r="J161" s="12">
-        <v>0</v>
+        <v>6931824.579999999</v>
       </c>
       <c r="K161" s="14">
-        <v>44767</v>
+        <v>44707</v>
       </c>
       <c r="L161" s="14">
-        <v>45411</v>
+        <v>45280</v>
       </c>
     </row>
     <row r="162" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A162" s="11" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B162" s="11" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="C162" s="11" t="s">
-        <v>136</v>
+        <v>249</v>
       </c>
       <c r="D162" s="11" t="s">
         <v>15</v>
       </c>
       <c r="E162" s="11" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="F162" s="11" t="s">
-        <v>57</v>
+        <v>149</v>
       </c>
       <c r="G162" s="11">
-        <v>0.9122</v>
+        <v>1</v>
       </c>
       <c r="H162" s="12">
-        <v>22472818</v>
+        <v>13792679.79</v>
       </c>
       <c r="I162" s="13">
-        <v>20500685.68</v>
+        <v>13792679.79</v>
       </c>
       <c r="J162" s="12">
-        <v>1972132.3200000003</v>
+        <v>0</v>
       </c>
       <c r="K162" s="14">
-        <v>44827</v>
+        <v>44767</v>
       </c>
       <c r="L162" s="14">
-        <v>45460</v>
+        <v>45411</v>
       </c>
     </row>
     <row r="163" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A163" s="11" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B163" s="11" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="C163" s="11" t="s">
-        <v>614</v>
+        <v>136</v>
       </c>
       <c r="D163" s="11" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="E163" s="11" t="s">
         <v>615</v>
       </c>
       <c r="F163" s="11" t="s">
-        <v>616</v>
+        <v>57</v>
       </c>
       <c r="G163" s="11">
-        <v>0.8996</v>
+        <v>0.9122</v>
       </c>
       <c r="H163" s="12">
-        <v>51414775.09</v>
+        <v>22472818</v>
       </c>
       <c r="I163" s="13">
-        <v>46254135.59</v>
+        <v>20500685.68</v>
       </c>
       <c r="J163" s="12">
-        <v>5160639.5</v>
+        <v>1972132.3200000003</v>
       </c>
       <c r="K163" s="14">
-        <v>45566</v>
+        <v>44827</v>
       </c>
       <c r="L163" s="14">
-        <v>46106</v>
+        <v>45460</v>
       </c>
     </row>
     <row r="164" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A164" s="11" t="s">
+        <v>611</v>
+      </c>
+      <c r="B164" s="11" t="s">
+        <v>616</v>
+      </c>
+      <c r="C164" s="11" t="s">
         <v>617</v>
-      </c>
-      <c r="B164" s="11" t="s">
-        <v>618</v>
-      </c>
-      <c r="C164" s="11" t="s">
-        <v>619</v>
       </c>
       <c r="D164" s="11" t="s">
         <v>34</v>
       </c>
       <c r="E164" s="11" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="F164" s="11" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="G164" s="11">
-        <v>0</v>
+        <v>0.8996</v>
       </c>
       <c r="H164" s="12">
-        <v>1302281.25</v>
+        <v>51414775.09</v>
       </c>
       <c r="I164" s="13">
-        <v>0</v>
+        <v>46254135.59</v>
       </c>
       <c r="J164" s="12">
-        <v>1302281.25</v>
+        <v>5160639.5</v>
       </c>
       <c r="K164" s="14">
-        <v>46080</v>
+        <v>45566</v>
       </c>
       <c r="L164" s="14">
-        <v>46440</v>
+        <v>46106</v>
       </c>
     </row>
     <row r="165" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A165" s="11" t="s">
+        <v>620</v>
+      </c>
+      <c r="B165" s="11" t="s">
+        <v>621</v>
+      </c>
+      <c r="C165" s="11" t="s">
         <v>622</v>
-      </c>
-      <c r="B165" s="11" t="s">
-        <v>623</v>
-      </c>
-      <c r="C165" s="11" t="s">
-        <v>161</v>
       </c>
       <c r="D165" s="11" t="s">
         <v>34</v>
       </c>
       <c r="E165" s="11" t="s">
+        <v>623</v>
+      </c>
+      <c r="F165" s="11" t="s">
         <v>624</v>
       </c>
-      <c r="F165" s="11" t="s">
-        <v>625</v>
-      </c>
       <c r="G165" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H165" s="12">
-        <v>18264452.89</v>
+        <v>1302281.25</v>
       </c>
       <c r="I165" s="13">
-        <v>18264452.89</v>
+        <v>0</v>
       </c>
       <c r="J165" s="12">
-        <v>0</v>
+        <v>1302281.25</v>
       </c>
       <c r="K165" s="14">
-        <v>44722</v>
+        <v>46080</v>
       </c>
       <c r="L165" s="14">
-        <v>45723</v>
+        <v>46440</v>
       </c>
     </row>
     <row r="166" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A166" s="11" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="B166" s="11" t="s">
         <v>626</v>
       </c>
       <c r="C166" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="D166" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E166" s="11" t="s">
         <v>627</v>
       </c>
-      <c r="D166" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="E166" s="11" t="s">
+      <c r="F166" s="11" t="s">
         <v>628</v>
       </c>
-      <c r="F166" s="11" t="s">
-        <v>40</v>
-      </c>
       <c r="G166" s="11">
-        <v>0.9953</v>
+        <v>1</v>
       </c>
       <c r="H166" s="12">
-        <v>30599999.01</v>
+        <v>18264452.89</v>
       </c>
       <c r="I166" s="13">
-        <v>30456294.33</v>
+        <v>18264452.89</v>
       </c>
       <c r="J166" s="12">
-        <v>143704.68000000343</v>
+        <v>0</v>
       </c>
       <c r="K166" s="14">
-        <v>45019</v>
+        <v>44722</v>
       </c>
       <c r="L166" s="14">
-        <v>45743</v>
+        <v>45723</v>
       </c>
     </row>
     <row r="167" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A167" s="11" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="B167" s="11" t="s">
         <v>629</v>
@@ -8725,36 +8736,36 @@
         <v>630</v>
       </c>
       <c r="D167" s="11" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="E167" s="11" t="s">
         <v>631</v>
       </c>
       <c r="F167" s="11" t="s">
-        <v>222</v>
+        <v>40</v>
       </c>
       <c r="G167" s="11">
-        <v>0.9601000000000001</v>
+        <v>0.9953</v>
       </c>
       <c r="H167" s="12">
-        <v>43796954.98</v>
+        <v>30599999.01</v>
       </c>
       <c r="I167" s="13">
-        <v>42048979.52</v>
+        <v>30456294.33</v>
       </c>
       <c r="J167" s="12">
-        <v>1747975.4599999934</v>
+        <v>143704.68000000343</v>
       </c>
       <c r="K167" s="14">
-        <v>44641</v>
+        <v>45019</v>
       </c>
       <c r="L167" s="14">
-        <v>46091</v>
+        <v>45743</v>
       </c>
     </row>
     <row r="168" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A168" s="11" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="B168" s="11" t="s">
         <v>632</v>
@@ -8772,27 +8783,27 @@
         <v>222</v>
       </c>
       <c r="G168" s="11">
-        <v>0.7956</v>
+        <v>0.9601000000000001</v>
       </c>
       <c r="H168" s="12">
-        <v>45726170.25</v>
+        <v>43796954.98</v>
       </c>
       <c r="I168" s="13">
-        <v>36377601.26</v>
+        <v>42048979.52</v>
       </c>
       <c r="J168" s="12">
-        <v>9348568.990000002</v>
+        <v>1747975.4599999934</v>
       </c>
       <c r="K168" s="14">
-        <v>44623</v>
+        <v>44641</v>
       </c>
       <c r="L168" s="14">
-        <v>46222</v>
+        <v>46091</v>
       </c>
     </row>
     <row r="169" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A169" s="11" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="B169" s="11" t="s">
         <v>635</v>
@@ -8807,24 +8818,62 @@
         <v>637</v>
       </c>
       <c r="F169" s="11" t="s">
-        <v>111</v>
+        <v>222</v>
       </c>
       <c r="G169" s="11">
-        <v>0.30670000000000003</v>
+        <v>0.7956</v>
       </c>
       <c r="H169" s="12">
-        <v>65678550.13</v>
+        <v>45726170.25</v>
       </c>
       <c r="I169" s="13">
-        <v>20145177.51</v>
+        <v>36377601.26</v>
       </c>
       <c r="J169" s="12">
-        <v>45533372.620000005</v>
+        <v>9348568.990000002</v>
       </c>
       <c r="K169" s="14">
         <v>44623</v>
       </c>
       <c r="L169" s="14">
+        <v>46222</v>
+      </c>
+    </row>
+    <row r="170" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A170" s="11" t="s">
+        <v>625</v>
+      </c>
+      <c r="B170" s="11" t="s">
+        <v>638</v>
+      </c>
+      <c r="C170" s="11" t="s">
+        <v>639</v>
+      </c>
+      <c r="D170" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E170" s="11" t="s">
+        <v>640</v>
+      </c>
+      <c r="F170" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="G170" s="11">
+        <v>0.30670000000000003</v>
+      </c>
+      <c r="H170" s="12">
+        <v>65678550.13</v>
+      </c>
+      <c r="I170" s="13">
+        <v>20145177.51</v>
+      </c>
+      <c r="J170" s="12">
+        <v>45533372.620000005</v>
+      </c>
+      <c r="K170" s="14">
+        <v>44623</v>
+      </c>
+      <c r="L170" s="14">
         <v>46170</v>
       </c>
     </row>

</xml_diff>